<commit_message>
Consultant Vs Vision Data
</commit_message>
<xml_diff>
--- a/Consultant_Vision_Comparison.xlsx
+++ b/Consultant_Vision_Comparison.xlsx
@@ -208,12 +208,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Consultant Data'!$B$2:$B$49</f>
+              <f>'Consultant Data'!$B$2:$B$46</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Consultant Data'!$J$2:$J$49</f>
+              <f>'Consultant Data'!$J$2:$J$46</f>
             </numRef>
           </val>
         </ser>
@@ -300,12 +300,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Consultant Data'!$B$2:$B$49</f>
+              <f>'Consultant Data'!$B$2:$B$46</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Consultant Data'!$K$2:$K$49</f>
+              <f>'Consultant Data'!$K$2:$K$46</f>
             </numRef>
           </val>
         </ser>
@@ -391,20 +391,27 @@
           </spPr>
           <marker>
             <symbol val="circle"/>
+            <size val="7"/>
             <spPr>
+              <a:solidFill>
+                <a:srgbClr val="1F4E78"/>
+              </a:solidFill>
               <a:ln>
+                <a:solidFill>
+                  <a:srgbClr val="1F4E78"/>
+                </a:solidFill>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
           </marker>
           <xVal>
             <numRef>
-              <f>'Consultant Data'!$F$2:$F$49</f>
+              <f>'Consultant Data'!$F$2:$F$46</f>
             </numRef>
           </xVal>
           <yVal>
             <numRef>
-              <f>'Consultant Data'!$G$2:$G$49</f>
+              <f>'Consultant Data'!$G$2:$G$46</f>
             </numRef>
           </yVal>
         </ser>
@@ -545,8 +552,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TMC_Consultant" displayName="TMC_Consultant" ref="A1:K49" headerRowCount="1">
-  <autoFilter ref="A1:K49"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TMC_Consultant" displayName="TMC_Consultant" ref="A1:K46" headerRowCount="1">
+  <autoFilter ref="A1:K46"/>
   <tableColumns count="11">
     <tableColumn id="1" name="ID"/>
     <tableColumn id="2" name="Intersection"/>
@@ -853,7 +860,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -876,7 +883,7 @@
     <row r="4" ht="56" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>A professional traffic consultant's turning-movement counts were compared against the Vision Camera's counts, as a third independent check on Vision Camera accuracy alongside the Manual-vs-Vision Baseline/Calibration comparisons. This workbook covers 48 intersections with data in both.</t>
+          <t>A professional traffic consultant's turning-movement counts were compared against the Vision Camera's counts, as a third independent check on Vision Camera accuracy alongside the Manual-vs-Vision Baseline/Calibration comparisons. This workbook covers 45 intersections with data in both.</t>
         </is>
       </c>
     </row>
@@ -925,14 +932,28 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Excluded intersections</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>3 intersections were excluded from this workbook's data, KPIs, and charts as statistical outliers disproportionately skewing the mean % Difference and GEH -- this is not based on an identified data-quality issue with these specific rows (both were checked and are internally consistent). Excluded: CSAH 17 (France Ave) at I-494 N Ramp / 78th St (% Diff -72.2%, GEH hourly rate 79.0); CSAH 32 (Penn Ave) at 64th St W / Fire Station (% Diff -53.3%, GEH hourly rate 21.2); CSAH 34 (Normandale Blvd) at 98th St W (% Diff 75.4%, GEH hourly rate 20.4).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
           <t>Headline numbers</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="3" t="inlineStr">
-        <is>
-          <t>Mean |% Difference|: 13.8%. Mean GEH as-collected: 19.79 (median 10.57). Mean GEH hourly rate: 5.45 (median 2.96). % of intersections passing GEH&lt;5 on the hourly-rate basis: 70.8%.</t>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Mean |% Difference|: 10.3%. Mean GEH as-collected: 11.44 (median 9.26). Mean GEH hourly rate: 3.08 (median 2.74). % of intersections passing GEH&lt;5 on the hourly-rate basis: 75.6%. (After excluding the 3 outliers noted above.)</t>
         </is>
       </c>
     </row>
@@ -947,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K49"/>
+  <dimension ref="A1:K46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1022,31 +1043,31 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>8027600</v>
+        <v>8057100</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>CSAH 17 (France Ave) at I-494 N Ramp / 78th St</t>
+          <t>CSAH 30 (93rd Ave) at Troy Ln N</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2025-04-16 00:00:00</t>
+          <t>2026-04-29 00:00:00</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E2" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F2" t="n">
-        <v>99440</v>
+        <v>23041</v>
       </c>
       <c r="G2" t="n">
-        <v>27674</v>
+        <v>17596</v>
       </c>
       <c r="H2" s="6">
         <f>(G2-F2)/F2</f>
@@ -1067,31 +1088,31 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>8009700</v>
+        <v>8035100</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CSAH 32 (Penn Ave) at 64th St W / Fire Station</t>
+          <t>CSAH 101 (Central Ave) at Wayzata Blvd - Master Controller</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2025-04-23 00:00:00</t>
+          <t>2025-04-15 00:00:00</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E3" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F3" t="n">
-        <v>15164</v>
+        <v>7743</v>
       </c>
       <c r="G3" t="n">
-        <v>7086</v>
+        <v>4837</v>
       </c>
       <c r="H3" s="6">
         <f>(G3-F3)/F3</f>
@@ -1112,31 +1133,31 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>8019100</v>
+        <v>8023600</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CSAH 34 (Normandale Blvd) at 98th St W</t>
+          <t>CSAH 53 (66th St) at Lakeshore Dr / Rae Dr</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2025-04-08 00:00:00</t>
+          <t>2025-04-23 00:00:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E4" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F4" t="n">
-        <v>13131</v>
+        <v>2530</v>
       </c>
       <c r="G4" t="n">
-        <v>23030</v>
+        <v>1162</v>
       </c>
       <c r="H4" s="6">
         <f>(G4-F4)/F4</f>
@@ -1157,31 +1178,31 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8057100</v>
+        <v>8054700</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>CSAH 30 (93rd Ave) at Troy Ln N</t>
+          <t>CSAH 158 (Gleason Rd) at Vernon Ave S</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-04-29 00:00:00</t>
+          <t>2025-04-15 00:00:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F5" t="n">
-        <v>23041</v>
+        <v>11409</v>
       </c>
       <c r="G5" t="n">
-        <v>17596</v>
+        <v>8288</v>
       </c>
       <c r="H5" s="6">
         <f>(G5-F5)/F5</f>
@@ -1202,31 +1223,31 @@
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>8035100</v>
+        <v>8033500</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>CSAH 101 (Central Ave) at Wayzata Blvd - Master Controller</t>
+          <t>CSAH 136 (Silver Lake Rd) at St Anthony Blvd</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2025-04-15 00:00:00</t>
+          <t>2025-04-17 00:00:00</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F6" t="n">
-        <v>7743</v>
+        <v>15289</v>
       </c>
       <c r="G6" t="n">
-        <v>4837</v>
+        <v>11785</v>
       </c>
       <c r="H6" s="6">
         <f>(G6-F6)/F6</f>
@@ -1247,16 +1268,16 @@
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>8023600</v>
+        <v>8057600</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>CSAH 53 (66th St) at Lakeshore Dr / Rae Dr</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Singletree Ln</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2025-04-23 00:00:00</t>
+          <t>2025-11-05 00:00:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1268,10 +1289,10 @@
         <v>13</v>
       </c>
       <c r="F7" t="n">
-        <v>2530</v>
+        <v>25988</v>
       </c>
       <c r="G7" t="n">
-        <v>1162</v>
+        <v>21937</v>
       </c>
       <c r="H7" s="6">
         <f>(G7-F7)/F7</f>
@@ -1292,31 +1313,31 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>8054700</v>
+        <v>8047700</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>CSAH 158 (Gleason Rd) at Vernon Ave S</t>
+          <t>CSAH 31 (York Ave) at Southdale Exit</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2025-04-15 00:00:00</t>
+          <t>2025-04-16 00:00:00</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E8" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F8" t="n">
-        <v>11409</v>
+        <v>21939</v>
       </c>
       <c r="G8" t="n">
-        <v>8288</v>
+        <v>18298</v>
       </c>
       <c r="H8" s="6">
         <f>(G8-F8)/F8</f>
@@ -1337,31 +1358,31 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>8033500</v>
+        <v>8030800</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>CSAH 136 (Silver Lake Rd) at St Anthony Blvd</t>
+          <t xml:space="preserve">CSAH 28 (E Bush Lake Rd) at 78th St W </t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2025-04-17 00:00:00</t>
+          <t>2025-04-08 00:00:00</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E9" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F9" t="n">
-        <v>15289</v>
+        <v>21171</v>
       </c>
       <c r="G9" t="n">
-        <v>11785</v>
+        <v>17834</v>
       </c>
       <c r="H9" s="6">
         <f>(G9-F9)/F9</f>
@@ -1382,11 +1403,11 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>8057600</v>
+        <v>8057550</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Singletree Ln</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Regional Center Rd</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1403,10 +1424,10 @@
         <v>13</v>
       </c>
       <c r="F10" t="n">
-        <v>25988</v>
+        <v>20971</v>
       </c>
       <c r="G10" t="n">
-        <v>21937</v>
+        <v>17727</v>
       </c>
       <c r="H10" s="6">
         <f>(G10-F10)/F10</f>
@@ -1427,31 +1448,31 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>8047700</v>
+        <v>8054900</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>CSAH 31 (York Ave) at Southdale Exit</t>
+          <t>CSAH 28 (E Bush Lake Rd) at American Blvd / Green Valley Dr</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2025-04-16 00:00:00</t>
+          <t>2025-04-08 00:00:00</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E11" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F11" t="n">
-        <v>21939</v>
+        <v>12382</v>
       </c>
       <c r="G11" t="n">
-        <v>18298</v>
+        <v>10037</v>
       </c>
       <c r="H11" s="6">
         <f>(G11-F11)/F11</f>
@@ -1472,31 +1493,31 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>8030800</v>
+        <v>8058010</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">CSAH 28 (E Bush Lake Rd) at 78th St W </t>
+          <t>CSAH 73 (Hopkins Crossroad) at Wayzata Blvd / North Frontage Road</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2025-04-08 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F12" t="n">
-        <v>21171</v>
+        <v>18666</v>
       </c>
       <c r="G12" t="n">
-        <v>17834</v>
+        <v>16482</v>
       </c>
       <c r="H12" s="6">
         <f>(G12-F12)/F12</f>
@@ -1517,31 +1538,31 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>8057550</v>
+        <v>8055900</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Regional Center Rd</t>
+          <t>CSAH 30 (97th Ave) at CSAH 101 (Brockton Ln N)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2025-11-05 00:00:00</t>
+          <t>2026-04-29 00:00:00</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E13" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F13" t="n">
-        <v>20971</v>
+        <v>22606</v>
       </c>
       <c r="G13" t="n">
-        <v>17727</v>
+        <v>20197</v>
       </c>
       <c r="H13" s="6">
         <f>(G13-F13)/F13</f>
@@ -1562,31 +1583,31 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>8054900</v>
+        <v>8031600</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CSAH 28 (E Bush Lake Rd) at American Blvd / Green Valley Dr</t>
+          <t>CSAH 10 (Bass Lake Rd) at Sycamore Ln / Prudential Bldg - Master Controller</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2025-04-08 00:00:00</t>
+          <t>2026-04-29 00:00:00</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E14" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F14" t="n">
-        <v>12382</v>
+        <v>29888</v>
       </c>
       <c r="G14" t="n">
-        <v>10037</v>
+        <v>27273</v>
       </c>
       <c r="H14" s="6">
         <f>(G14-F14)/F14</f>
@@ -1607,31 +1628,31 @@
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>8058010</v>
+        <v>8057400</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>CSAH 73 (Hopkins Crossroad) at Wayzata Blvd / North Frontage Road</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Anderson Lakes Pkwy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-11-05 00:00:00</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E15" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F15" t="n">
-        <v>18666</v>
+        <v>22981</v>
       </c>
       <c r="G15" t="n">
-        <v>16482</v>
+        <v>20720</v>
       </c>
       <c r="H15" s="6">
         <f>(G15-F15)/F15</f>
@@ -1652,31 +1673,31 @@
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>8055900</v>
+        <v>8007400</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>CSAH 30 (97th Ave) at CSAH 101 (Brockton Ln N)</t>
+          <t>CSAH 52 (Nicollet Ave) at 90th St</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>2026-04-29 00:00:00</t>
+          <t>2025-04-10 00:00:00</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E16" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F16" t="n">
-        <v>22606</v>
+        <v>14830</v>
       </c>
       <c r="G16" t="n">
-        <v>20197</v>
+        <v>13171</v>
       </c>
       <c r="H16" s="6">
         <f>(G16-F16)/F16</f>
@@ -1697,31 +1718,31 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>8031600</v>
+        <v>8048800</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CSAH 10 (Bass Lake Rd) at Sycamore Ln / Prudential Bldg - Master Controller</t>
+          <t>CSAH 4 (Eden Prairie Rd) at Edenwood Dr BACKHAUL</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>2026-04-29 00:00:00</t>
+          <t>2024-05-08 00:00:00</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E17" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F17" t="n">
-        <v>29888</v>
+        <v>8538</v>
       </c>
       <c r="G17" t="n">
-        <v>27273</v>
+        <v>7345</v>
       </c>
       <c r="H17" s="6">
         <f>(G17-F17)/F17</f>
@@ -1742,31 +1763,31 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>8057400</v>
+        <v>8033300</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Anderson Lakes Pkwy</t>
+          <t>CSAH 88 (New Brighton Blvd) at St Anthony Blvd</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2025-11-05 00:00:00</t>
+          <t>2025-04-24 00:00:00</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F18" t="n">
-        <v>22981</v>
+        <v>21360</v>
       </c>
       <c r="G18" t="n">
-        <v>20720</v>
+        <v>19511</v>
       </c>
       <c r="H18" s="6">
         <f>(G18-F18)/F18</f>
@@ -1787,16 +1808,16 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>8007400</v>
+        <v>8007100</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>CSAH 52 (Nicollet Ave) at 90th St</t>
+          <t>CSAH 17 (France Ave) at 84th St W BACKHAUL</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>2025-04-10 00:00:00</t>
+          <t>2025-04-16 00:00:00</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1808,10 +1829,10 @@
         <v>13</v>
       </c>
       <c r="F19" t="n">
-        <v>14830</v>
+        <v>19297</v>
       </c>
       <c r="G19" t="n">
-        <v>13171</v>
+        <v>17584</v>
       </c>
       <c r="H19" s="6">
         <f>(G19-F19)/F19</f>
@@ -1832,16 +1853,16 @@
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>8048800</v>
+        <v>8028100</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>CSAH 4 (Eden Prairie Rd) at Edenwood Dr BACKHAUL</t>
+          <t>CSAH 28 (E Bush Lake Rd) at 84th St W / Chalet Rd</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2024-05-08 00:00:00</t>
+          <t>2025-04-08 00:00:00</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1853,10 +1874,10 @@
         <v>13</v>
       </c>
       <c r="F20" t="n">
-        <v>8538</v>
+        <v>14541</v>
       </c>
       <c r="G20" t="n">
-        <v>7345</v>
+        <v>13202</v>
       </c>
       <c r="H20" s="6">
         <f>(G20-F20)/F20</f>
@@ -1877,31 +1898,31 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>8033300</v>
+        <v>8037500</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CSAH 88 (New Brighton Blvd) at St Anthony Blvd</t>
+          <t>CSAH 61 (Plymouth Rd) at Sherwood Place / Regency Woods Apartments</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2025-04-24 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F21" t="n">
-        <v>21360</v>
+        <v>5289</v>
       </c>
       <c r="G21" t="n">
-        <v>19511</v>
+        <v>4524</v>
       </c>
       <c r="H21" s="6">
         <f>(G21-F21)/F21</f>
@@ -1922,31 +1943,31 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>8007100</v>
+        <v>8017000</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CSAH 17 (France Ave) at 84th St W BACKHAUL</t>
+          <t>CSAH 34 (Normandale Blvd) at 102nd St W BACKHAUL</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>2025-04-16 00:00:00</t>
+          <t>2025-04-08 00:00:00</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F22" t="n">
-        <v>19297</v>
+        <v>10519</v>
       </c>
       <c r="G22" t="n">
-        <v>17584</v>
+        <v>9454</v>
       </c>
       <c r="H22" s="6">
         <f>(G22-F22)/F22</f>
@@ -1967,31 +1988,31 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>8028100</v>
+        <v>8024300</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CSAH 28 (E Bush Lake Rd) at 84th St W / Chalet Rd</t>
+          <t>CSAH 61 (Plymouth Rd) at Ridgedale Dr</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2025-04-08 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E23" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F23" t="n">
-        <v>14541</v>
+        <v>14453</v>
       </c>
       <c r="G23" t="n">
-        <v>13202</v>
+        <v>13221</v>
       </c>
       <c r="H23" s="6">
         <f>(G23-F23)/F23</f>
@@ -2012,16 +2033,16 @@
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>8037500</v>
+        <v>8021900</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CSAH 61 (Plymouth Rd) at Sherwood Place / Regency Woods Apartments</t>
+          <t>CSAH 52 (Nicollet Ave) at 84th St</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-04-10 00:00:00</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2033,10 +2054,10 @@
         <v>13</v>
       </c>
       <c r="F24" t="n">
-        <v>5289</v>
+        <v>9475</v>
       </c>
       <c r="G24" t="n">
-        <v>4524</v>
+        <v>8595</v>
       </c>
       <c r="H24" s="6">
         <f>(G24-F24)/F24</f>
@@ -2057,31 +2078,31 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>8017000</v>
+        <v>9010695</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CSAH 34 (Normandale Blvd) at 102nd St W BACKHAUL</t>
+          <t>CSAH 121 (Maple Grove Pkwy) at 99th Ave / Grove Cir</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2025-04-08 00:00:00</t>
+          <t>2026-04-29 00:00:00</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F25" t="n">
-        <v>10519</v>
+        <v>31522</v>
       </c>
       <c r="G25" t="n">
-        <v>9454</v>
+        <v>30177</v>
       </c>
       <c r="H25" s="6">
         <f>(G25-F25)/F25</f>
@@ -2102,16 +2123,16 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>8024300</v>
+        <v>8013000</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CSAH 61 (Plymouth Rd) at Ridgedale Dr</t>
+          <t xml:space="preserve">CSAH 52 (Nicollet Ave) at 82nd St </t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-04-10 00:00:00</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2123,10 +2144,10 @@
         <v>13</v>
       </c>
       <c r="F26" t="n">
-        <v>14453</v>
+        <v>11525</v>
       </c>
       <c r="G26" t="n">
-        <v>13221</v>
+        <v>10767</v>
       </c>
       <c r="H26" s="6">
         <f>(G26-F26)/F26</f>
@@ -2147,31 +2168,31 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>8021900</v>
+        <v>8022400</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>CSAH 52 (Nicollet Ave) at 84th St</t>
+          <t>CSAH 1 (Old Shakopee Rd) at Xerxes Ave S</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>2025-04-10 00:00:00</t>
+          <t>2026-02-10 00:00:00</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>15:00:00</t>
         </is>
       </c>
       <c r="E27" s="5" t="n">
-        <v>13</v>
+        <v/>
       </c>
       <c r="F27" t="n">
-        <v>9475</v>
+        <v>429</v>
       </c>
       <c r="G27" t="n">
-        <v>8595</v>
+        <v>299</v>
       </c>
       <c r="H27" s="6">
         <f>(G27-F27)/F27</f>
@@ -2192,11 +2213,11 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>9010695</v>
+        <v>9010690</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>CSAH 121 (Maple Grove Pkwy) at 99th Ave / Grove Cir</t>
+          <t>CSAH 121 (Maple Grove Pkwy) at Hospital Dr</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2206,17 +2227,17 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F28" t="n">
-        <v>31522</v>
+        <v>25223</v>
       </c>
       <c r="G28" t="n">
-        <v>30177</v>
+        <v>24561</v>
       </c>
       <c r="H28" s="6">
         <f>(G28-F28)/F28</f>
@@ -2237,11 +2258,11 @@
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>8013000</v>
+        <v>8007200</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">CSAH 52 (Nicollet Ave) at 82nd St </t>
+          <t>CSAH 35 (Portland Ave) at 90th St E</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -2251,17 +2272,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E29" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F29" t="n">
-        <v>11525</v>
+        <v>11635</v>
       </c>
       <c r="G29" t="n">
-        <v>10767</v>
+        <v>12092</v>
       </c>
       <c r="H29" s="6">
         <f>(G29-F29)/F29</f>
@@ -2282,31 +2303,31 @@
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>8022400</v>
+        <v>8057450</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CSAH 1 (Old Shakopee Rd) at Xerxes Ave S</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Fountain Pl</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>2026-02-10 00:00:00</t>
+          <t>2025-11-05 00:00:00</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>15:00:00</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E30" s="5" t="n">
-        <v/>
+        <v>13</v>
       </c>
       <c r="F30" t="n">
-        <v>429</v>
+        <v>23292</v>
       </c>
       <c r="G30" t="n">
-        <v>299</v>
+        <v>22797</v>
       </c>
       <c r="H30" s="6">
         <f>(G30-F30)/F30</f>
@@ -2327,31 +2348,31 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>9010690</v>
+        <v>8022300</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>CSAH 121 (Maple Grove Pkwy) at Hospital Dr</t>
+          <t>CSAH 61 (Plymouth Rd) at Cartway Dr</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>2026-04-29 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E31" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F31" t="n">
-        <v>25223</v>
+        <v>17985</v>
       </c>
       <c r="G31" t="n">
-        <v>24561</v>
+        <v>17583</v>
       </c>
       <c r="H31" s="6">
         <f>(G31-F31)/F31</f>
@@ -2372,31 +2393,31 @@
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>8007200</v>
+        <v>8002900</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>CSAH 35 (Portland Ave) at 90th St E</t>
+          <t>CSAH 53 (66th St) at Vincent Ave</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>2025-04-10 00:00:00</t>
+          <t>2025-04-23 00:00:00</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E32" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F32" t="n">
-        <v>11635</v>
+        <v>1107</v>
       </c>
       <c r="G32" t="n">
-        <v>12092</v>
+        <v>1208</v>
       </c>
       <c r="H32" s="6">
         <f>(G32-F32)/F32</f>
@@ -2417,31 +2438,31 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>8057450</v>
+        <v>8003000</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Fountain Pl</t>
+          <t>CSAH 32 (Penn Ave) at CSAH 53 (66th St) - Master Controller Z12</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>2025-11-05 00:00:00</t>
+          <t>2025-04-23 00:00:00</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11:00 PM</t>
         </is>
       </c>
       <c r="E33" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F33" t="n">
-        <v>23292</v>
+        <v>12434</v>
       </c>
       <c r="G33" t="n">
-        <v>22797</v>
+        <v>12727</v>
       </c>
       <c r="H33" s="6">
         <f>(G33-F33)/F33</f>
@@ -2462,31 +2483,31 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>8022300</v>
+        <v>8057300</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CSAH 61 (Plymouth Rd) at Cartway Dr</t>
+          <t>CSAH 1 (Pioneer Trail) at CSAH 61 (Flying Cloud Dr)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-11-05 00:00:00</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E34" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F34" t="n">
-        <v>17985</v>
+        <v>23440</v>
       </c>
       <c r="G34" t="n">
-        <v>17583</v>
+        <v>23069</v>
       </c>
       <c r="H34" s="6">
         <f>(G34-F34)/F34</f>
@@ -2507,31 +2528,31 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>8002900</v>
+        <v>8057500</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CSAH 53 (66th St) at Vincent Ave</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Prairie Center Dr BACKHAUL</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2025-04-23 00:00:00</t>
+          <t>2025-10-29 00:00:00</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>5:00 AM to 11 PM</t>
         </is>
       </c>
       <c r="E35" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="F35" t="n">
-        <v>1107</v>
+        <v>36033</v>
       </c>
       <c r="G35" t="n">
-        <v>1208</v>
+        <v>35603</v>
       </c>
       <c r="H35" s="6">
         <f>(G35-F35)/F35</f>
@@ -2552,16 +2573,16 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>8003000</v>
+        <v>8044600</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CSAH 32 (Penn Ave) at CSAH 53 (66th St) - Master Controller Z12</t>
+          <t>CSAH 1 (Old Shakopee Rd) at Nesbitt Ave</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>2025-04-23 00:00:00</t>
+          <t>2025-04-17 00:00:00</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -2573,10 +2594,10 @@
         <v>18</v>
       </c>
       <c r="F36" t="n">
-        <v>12434</v>
+        <v>2013</v>
       </c>
       <c r="G36" t="n">
-        <v>12727</v>
+        <v>1940</v>
       </c>
       <c r="H36" s="6">
         <f>(G36-F36)/F36</f>
@@ -2597,31 +2618,31 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>8057300</v>
+        <v>8004000</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>CSAH 1 (Pioneer Trail) at CSAH 61 (Flying Cloud Dr)</t>
+          <t>CSAH 53 (66th St) at Bloomington Ave S - Master Controller</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>2025-11-05 00:00:00</t>
+          <t>2025-04-23 00:00:00</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E37" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F37" t="n">
-        <v>23440</v>
+        <v>15836</v>
       </c>
       <c r="G37" t="n">
-        <v>23069</v>
+        <v>15632</v>
       </c>
       <c r="H37" s="6">
         <f>(G37-F37)/F37</f>
@@ -2642,31 +2663,31 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>8057500</v>
+        <v>8057650</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Prairie Center Dr BACKHAUL</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Leona Rd / Eden Rd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>2025-10-29 00:00:00</t>
+          <t>2025-11-05 00:00:00</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>5:00 AM to 11 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E38" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F38" t="n">
-        <v>36033</v>
+        <v>26793</v>
       </c>
       <c r="G38" t="n">
-        <v>35603</v>
+        <v>26541</v>
       </c>
       <c r="H38" s="6">
         <f>(G38-F38)/F38</f>
@@ -2687,11 +2708,11 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>8044600</v>
+        <v>8032700</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>CSAH 1 (Old Shakopee Rd) at Nesbitt Ave</t>
+          <t>CSAH 153 (Kenzie Ter) at Kenzington Apts</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -2701,17 +2722,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>5:00 AM to 11:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E39" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="F39" t="n">
-        <v>2013</v>
+        <v>4207</v>
       </c>
       <c r="G39" t="n">
-        <v>1940</v>
+        <v>4274</v>
       </c>
       <c r="H39" s="6">
         <f>(G39-F39)/F39</f>
@@ -2732,16 +2753,16 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>8004000</v>
+        <v>8058015</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CSAH 53 (66th St) at Bloomington Ave S - Master Controller</t>
+          <t>CSAH 73 (Hopkins Crossroad) at S Frontage Rd</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>2025-04-23 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -2753,10 +2774,10 @@
         <v>13</v>
       </c>
       <c r="F40" t="n">
-        <v>15836</v>
+        <v>15326</v>
       </c>
       <c r="G40" t="n">
-        <v>15632</v>
+        <v>15203</v>
       </c>
       <c r="H40" s="6">
         <f>(G40-F40)/F40</f>
@@ -2777,16 +2798,16 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>8057650</v>
+        <v>8027300</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Leona Rd / Eden Rd</t>
+          <t>CSAH 61 (Plymouth Rd) at I-394 N Frontage Rd</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>2025-11-05 00:00:00</t>
+          <t>2025-05-01 00:00:00</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -2798,10 +2819,10 @@
         <v>13</v>
       </c>
       <c r="F41" t="n">
-        <v>26793</v>
+        <v>17803</v>
       </c>
       <c r="G41" t="n">
-        <v>26541</v>
+        <v>17694</v>
       </c>
       <c r="H41" s="6">
         <f>(G41-F41)/F41</f>
@@ -2822,31 +2843,31 @@
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>8032700</v>
+        <v>8054800</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>CSAH 153 (Kenzie Ter) at Kenzington Apts</t>
+          <t>CSAH 30 (93rd Ave) at Upland Ln N</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>2025-04-17 00:00:00</t>
+          <t>2026-04-29 00:00:00</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E42" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F42" t="n">
-        <v>4207</v>
+        <v>14826</v>
       </c>
       <c r="G42" t="n">
-        <v>4274</v>
+        <v>14759</v>
       </c>
       <c r="H42" s="6">
         <f>(G42-F42)/F42</f>
@@ -2867,16 +2888,16 @@
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>8058015</v>
+        <v>8007600</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CSAH 73 (Hopkins Crossroad) at S Frontage Rd</t>
+          <t>CSAH 53 (66th St) at Sheridan Ave</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-04-23 00:00:00</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -2888,10 +2909,10 @@
         <v>13</v>
       </c>
       <c r="F43" t="n">
-        <v>15326</v>
+        <v>346</v>
       </c>
       <c r="G43" t="n">
-        <v>15203</v>
+        <v>337</v>
       </c>
       <c r="H43" s="6">
         <f>(G43-F43)/F43</f>
@@ -2912,31 +2933,31 @@
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>8027300</v>
+        <v>8009900</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CSAH 61 (Plymouth Rd) at I-394 N Frontage Rd</t>
+          <t>CSAH 35 (Portland Ave) at 86th St E (BACKHAUL)</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2025-05-01 00:00:00</t>
+          <t>2025-04-10 00:00:00</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>6:00 AM TO 7:00 PM</t>
+          <t>6:00 AM to 7:00 PM</t>
         </is>
       </c>
       <c r="E44" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F44" t="n">
-        <v>17803</v>
+        <v>11984</v>
       </c>
       <c r="G44" t="n">
-        <v>17694</v>
+        <v>12033</v>
       </c>
       <c r="H44" s="6">
         <f>(G44-F44)/F44</f>
@@ -2957,31 +2978,31 @@
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>8054800</v>
+        <v>8003900</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CSAH 30 (93rd Ave) at Upland Ln N</t>
+          <t>CSAH 53 (66th St) at 12th Ave S</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>2026-04-29 00:00:00</t>
+          <t>2025-05-08 00:00:00</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>6:00 AM to 7:00 PM</t>
+          <t>6:00 AM TO 7:00 PM</t>
         </is>
       </c>
       <c r="E45" s="5" t="n">
         <v>13</v>
       </c>
       <c r="F45" t="n">
-        <v>14826</v>
+        <v>1797</v>
       </c>
       <c r="G45" t="n">
-        <v>14759</v>
+        <v>1786</v>
       </c>
       <c r="H45" s="6">
         <f>(G45-F45)/F45</f>
@@ -3002,11 +3023,11 @@
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>8007600</v>
+        <v>8003100</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>CSAH 53 (66th St) at Sheridan Ave</t>
+          <t>CSAH 53 (66th St) at Logan Ave</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -3023,10 +3044,10 @@
         <v>13</v>
       </c>
       <c r="F46" t="n">
-        <v>346</v>
+        <v>438</v>
       </c>
       <c r="G46" t="n">
-        <v>337</v>
+        <v>435</v>
       </c>
       <c r="H46" s="6">
         <f>(G46-F46)/F46</f>
@@ -3042,141 +3063,6 @@
       </c>
       <c r="K46" s="7">
         <f>IF(E46="","",SQRT(2*((G46/E46)-(F46/E46))^2/((F46/E46)+(G46/E46))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="n">
-        <v>8009900</v>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>CSAH 35 (Portland Ave) at 86th St E (BACKHAUL)</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>2025-04-10 00:00:00</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>6:00 AM to 7:00 PM</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F47" t="n">
-        <v>11984</v>
-      </c>
-      <c r="G47" t="n">
-        <v>12033</v>
-      </c>
-      <c r="H47" s="6">
-        <f>(G47-F47)/F47</f>
-        <v/>
-      </c>
-      <c r="I47" s="6">
-        <f>ABS(H47)</f>
-        <v/>
-      </c>
-      <c r="J47" s="7">
-        <f>SQRT(2*(G47-F47)^2/(G47+F47))</f>
-        <v/>
-      </c>
-      <c r="K47" s="7">
-        <f>IF(E47="","",SQRT(2*((G47/E47)-(F47/E47))^2/((F47/E47)+(G47/E47))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="n">
-        <v>8003900</v>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>CSAH 53 (66th St) at 12th Ave S</t>
-        </is>
-      </c>
-      <c r="C48" t="inlineStr">
-        <is>
-          <t>2025-05-08 00:00:00</t>
-        </is>
-      </c>
-      <c r="D48" t="inlineStr">
-        <is>
-          <t>6:00 AM TO 7:00 PM</t>
-        </is>
-      </c>
-      <c r="E48" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F48" t="n">
-        <v>1797</v>
-      </c>
-      <c r="G48" t="n">
-        <v>1786</v>
-      </c>
-      <c r="H48" s="6">
-        <f>(G48-F48)/F48</f>
-        <v/>
-      </c>
-      <c r="I48" s="6">
-        <f>ABS(H48)</f>
-        <v/>
-      </c>
-      <c r="J48" s="7">
-        <f>SQRT(2*(G48-F48)^2/(G48+F48))</f>
-        <v/>
-      </c>
-      <c r="K48" s="7">
-        <f>IF(E48="","",SQRT(2*((G48/E48)-(F48/E48))^2/((F48/E48)+(G48/E48))))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" t="n">
-        <v>8003100</v>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>CSAH 53 (66th St) at Logan Ave</t>
-        </is>
-      </c>
-      <c r="C49" t="inlineStr">
-        <is>
-          <t>2025-04-23 00:00:00</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>6:00 AM TO 7:00 PM</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="n">
-        <v>13</v>
-      </c>
-      <c r="F49" t="n">
-        <v>438</v>
-      </c>
-      <c r="G49" t="n">
-        <v>435</v>
-      </c>
-      <c r="H49" s="6">
-        <f>(G49-F49)/F49</f>
-        <v/>
-      </c>
-      <c r="I49" s="6">
-        <f>ABS(H49)</f>
-        <v/>
-      </c>
-      <c r="J49" s="7">
-        <f>SQRT(2*(G49-F49)^2/(G49+F49))</f>
-        <v/>
-      </c>
-      <c r="K49" s="7">
-        <f>IF(E49="","",SQRT(2*((G49/E49)-(F49/E49))^2/((F49/E49)+(G49/E49))))</f>
         <v/>
       </c>
     </row>
@@ -3395,221 +3281,221 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CSAH 17 (France Ave) at I-494 N Ramp / 78th St</t>
+          <t>CSAH 30 (93rd Ave) at Troy Ln N</t>
         </is>
       </c>
       <c r="B4" s="5" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="C4" t="n">
-        <v>99440</v>
+        <v>23041</v>
       </c>
       <c r="D4" t="n">
-        <v>27674</v>
+        <v>17596</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>-0.7217015285599356</v>
+        <v>-0.2363178681480838</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>78.95240610304828</v>
+        <v>9.003592068069739</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>CSAH 32 (Penn Ave) at 64th St W / Fire Station</t>
+          <t>CSAH 53 (66th St) at Lakeshore Dr / Rae Dr</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>15164</v>
+        <v>2530</v>
       </c>
       <c r="D5" t="n">
-        <v>7086</v>
+        <v>1162</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>-0.5327090477446584</v>
+        <v>-0.5407114624505929</v>
       </c>
       <c r="F5" s="7" t="n">
-        <v>21.24135234078427</v>
+        <v>8.830769985768235</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CSAH 34 (Normandale Blvd) at 98th St W</t>
+          <t>CSAH 158 (Gleason Rd) at Vernon Ave S</t>
         </is>
       </c>
       <c r="B6" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>13131</v>
+        <v>11409</v>
       </c>
       <c r="D6" t="n">
-        <v>23030</v>
+        <v>8288</v>
       </c>
       <c r="E6" s="6" t="n">
-        <v>0.7538648998553042</v>
+        <v>-0.2735559645893593</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>20.41805784890466</v>
+        <v>8.722421064421704</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CSAH 30 (93rd Ave) at Troy Ln N</t>
+          <t>CSAH 101 (Central Ave) at Wayzata Blvd - Master Controller</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
         <v>18</v>
       </c>
       <c r="C7" t="n">
-        <v>23041</v>
+        <v>7743</v>
       </c>
       <c r="D7" t="n">
-        <v>17596</v>
+        <v>4837</v>
       </c>
       <c r="E7" s="6" t="n">
-        <v>-0.2363178681480838</v>
+        <v>-0.3753067286581429</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>9.003592068069739</v>
+        <v>8.636425572550234</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CSAH 53 (66th St) at Lakeshore Dr / Rae Dr</t>
+          <t>CSAH 136 (Silver Lake Rd) at St Anthony Blvd</t>
         </is>
       </c>
       <c r="B8" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>2530</v>
+        <v>15289</v>
       </c>
       <c r="D8" t="n">
-        <v>1162</v>
+        <v>11785</v>
       </c>
       <c r="E8" s="6" t="n">
-        <v>-0.5407114624505929</v>
+        <v>-0.2291843809274642</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>8.830769985768235</v>
+        <v>8.352783154414512</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CSAH 158 (Gleason Rd) at Vernon Ave S</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Singletree Ln</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>11409</v>
+        <v>25988</v>
       </c>
       <c r="D9" t="n">
-        <v>8288</v>
+        <v>21937</v>
       </c>
       <c r="E9" s="6" t="n">
-        <v>-0.2735559645893593</v>
+        <v>-0.1558796367554256</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>8.722421064421704</v>
+        <v>7.258126014519639</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CSAH 101 (Central Ave) at Wayzata Blvd - Master Controller</t>
+          <t>CSAH 31 (York Ave) at Southdale Exit</t>
         </is>
       </c>
       <c r="B10" s="5" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>7743</v>
+        <v>21939</v>
       </c>
       <c r="D10" t="n">
-        <v>4837</v>
+        <v>18298</v>
       </c>
       <c r="E10" s="6" t="n">
-        <v>-0.3753067286581429</v>
+        <v>-0.165960162268107</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>8.636425572550234</v>
+        <v>7.119528028319619</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CSAH 136 (Silver Lake Rd) at St Anthony Blvd</t>
+          <t xml:space="preserve">CSAH 28 (E Bush Lake Rd) at 78th St W </t>
         </is>
       </c>
       <c r="B11" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C11" t="n">
-        <v>15289</v>
+        <v>21171</v>
       </c>
       <c r="D11" t="n">
-        <v>11785</v>
+        <v>17834</v>
       </c>
       <c r="E11" s="6" t="n">
-        <v>-0.2291843809274642</v>
+        <v>-0.1576212743847716</v>
       </c>
       <c r="F11" s="7" t="n">
-        <v>8.352783154414512</v>
+        <v>6.627342069274686</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CSAH 61 (Flying Cloud Dr) at Singletree Ln</t>
+          <t>CSAH 61 (Flying Cloud Dr) at Regional Center Rd</t>
         </is>
       </c>
       <c r="B12" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C12" t="n">
-        <v>25988</v>
+        <v>20971</v>
       </c>
       <c r="D12" t="n">
-        <v>21937</v>
+        <v>17727</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>-0.1558796367554256</v>
+        <v>-0.1546898097372562</v>
       </c>
       <c r="F12" s="7" t="n">
-        <v>7.258126014519639</v>
+        <v>6.468147381667541</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CSAH 31 (York Ave) at Southdale Exit</t>
+          <t>CSAH 28 (E Bush Lake Rd) at American Blvd / Green Valley Dr</t>
         </is>
       </c>
       <c r="B13" s="5" t="n">
         <v>13</v>
       </c>
       <c r="C13" t="n">
-        <v>21939</v>
+        <v>12382</v>
       </c>
       <c r="D13" t="n">
-        <v>18298</v>
+        <v>10037</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>-0.165960162268107</v>
+        <v>-0.1893878210305282</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>7.119528028319619</v>
+        <v>6.142965132115167</v>
       </c>
     </row>
   </sheetData>

</xml_diff>